<commit_message>
Restyle mapping-study figures for journal publication.
Use Times New Roman typography, colorblind-safe palette, panel labels, and annotated Fig05 improvement values.
</commit_message>
<xml_diff>
--- a/mapping study graphs/outputs/mahalanobis_greedy_vs_hungarian/tables/mahalanobis_greedy_vs_hungarian_tables.xlsx
+++ b/mapping study graphs/outputs/mahalanobis_greedy_vs_hungarian/tables/mahalanobis_greedy_vs_hungarian_tables.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2435,25 +2435,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.550131147570549</v>
+        <v>3.6759</v>
       </c>
       <c r="E43" t="n">
-        <v>2.062422642354435</v>
+        <v>3.3891</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.4877085052161139</v>
+        <v>-0.2867999999999999</v>
       </c>
       <c r="G43" t="n">
-        <v>-19.12484013540804</v>
+        <v>-7.802170896923201</v>
       </c>
       <c r="H43" t="b">
         <v>0</v>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>6497</v>
+        <v>1000</v>
       </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -2482,25 +2482,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2.167596417725627</v>
+        <v>3.3377</v>
       </c>
       <c r="E44" t="n">
-        <v>2.011109817987401</v>
+        <v>3.1203</v>
       </c>
       <c r="F44" t="n">
-        <v>-0.1564865997382263</v>
+        <v>-0.2174</v>
       </c>
       <c r="G44" t="n">
-        <v>-7.219360507267377</v>
+        <v>-6.513467357761334</v>
       </c>
       <c r="H44" t="b">
         <v>0</v>
@@ -2511,7 +2511,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>6497</v>
+        <v>1000</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
@@ -2529,25 +2529,25 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3.6759</v>
+        <v>5.4729</v>
       </c>
       <c r="E45" t="n">
-        <v>3.3891</v>
+        <v>5.1842</v>
       </c>
       <c r="F45" t="n">
-        <v>-0.2867999999999999</v>
+        <v>-0.2887000000000004</v>
       </c>
       <c r="G45" t="n">
-        <v>-7.802170896923201</v>
+        <v>-5.275082680114754</v>
       </c>
       <c r="H45" t="b">
         <v>0</v>
@@ -2571,30 +2571,30 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Wine</t>
+          <t>CDC</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3.3377</v>
+        <v>2.7934</v>
       </c>
       <c r="E46" t="n">
-        <v>3.1203</v>
+        <v>2.6942</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.2174</v>
+        <v>-0.09920000000000018</v>
       </c>
       <c r="G46" t="n">
-        <v>-6.513467357761334</v>
+        <v>-3.551227894322337</v>
       </c>
       <c r="H46" t="b">
         <v>0</v>
@@ -2618,30 +2618,30 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wine</t>
+          <t>CDC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>3.501071108209549</v>
+        <v>3.0372</v>
       </c>
       <c r="E47" t="n">
-        <v>3.096475460767122</v>
+        <v>2.801934</v>
       </c>
       <c r="F47" t="n">
-        <v>-0.4045956474424273</v>
+        <v>-0.2352659999999998</v>
       </c>
       <c r="G47" t="n">
-        <v>-11.55633904417719</v>
+        <v>-7.74614776768075</v>
       </c>
       <c r="H47" t="b">
         <v>0</v>
@@ -2652,7 +2652,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>6497</v>
+        <v>5000</v>
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
@@ -2665,30 +2665,30 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Wine</t>
+          <t>CDC</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5.4729</v>
+        <v>3.956109</v>
       </c>
       <c r="E48" t="n">
-        <v>5.1842</v>
+        <v>3.569087</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.2887000000000004</v>
+        <v>-0.387022</v>
       </c>
       <c r="G48" t="n">
-        <v>-5.275082680114754</v>
+        <v>-9.782895264008145</v>
       </c>
       <c r="H48" t="b">
         <v>0</v>
@@ -2699,7 +2699,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -2712,30 +2712,30 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Wine</t>
+          <t>CDC</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3.171785053292916</v>
+        <v>3.9642</v>
       </c>
       <c r="E49" t="n">
-        <v>2.740441860745499</v>
+        <v>3.8121</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.4313431925474172</v>
+        <v>-0.1520999999999999</v>
       </c>
       <c r="G49" t="n">
-        <v>-13.59938284908685</v>
+        <v>-3.836839715453304</v>
       </c>
       <c r="H49" t="b">
         <v>0</v>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>6497</v>
+        <v>1000</v>
       </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -2764,25 +2764,25 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2.7934</v>
+        <v>6.856</v>
       </c>
       <c r="E50" t="n">
-        <v>2.6942</v>
+        <v>6.7014</v>
       </c>
       <c r="F50" t="n">
-        <v>-0.09920000000000018</v>
+        <v>-0.1546000000000003</v>
       </c>
       <c r="G50" t="n">
-        <v>-3.551227894322337</v>
+        <v>-2.254959159859981</v>
       </c>
       <c r="H50" t="b">
         <v>0</v>
@@ -2811,25 +2811,25 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3.0372</v>
+        <v>3.446302</v>
       </c>
       <c r="E51" t="n">
-        <v>2.801934</v>
+        <v>3.072402</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.2352659999999998</v>
+        <v>-0.3739000000000003</v>
       </c>
       <c r="G51" t="n">
-        <v>-7.74614776768075</v>
+        <v>-10.84931036223756</v>
       </c>
       <c r="H51" t="b">
         <v>0</v>
@@ -2858,25 +2858,25 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3.956109</v>
+        <v>8.513500000000001</v>
       </c>
       <c r="E52" t="n">
-        <v>3.569087</v>
+        <v>8.3148</v>
       </c>
       <c r="F52" t="n">
-        <v>-0.387022</v>
+        <v>-0.1987000000000005</v>
       </c>
       <c r="G52" t="n">
-        <v>-9.782895264008145</v>
+        <v>-2.333940212603518</v>
       </c>
       <c r="H52" t="b">
         <v>0</v>
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
@@ -2905,25 +2905,25 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3.9642</v>
+        <v>3.788867</v>
       </c>
       <c r="E53" t="n">
-        <v>3.8121</v>
+        <v>3.345442</v>
       </c>
       <c r="F53" t="n">
-        <v>-0.1520999999999999</v>
+        <v>-0.4434250000000004</v>
       </c>
       <c r="G53" t="n">
-        <v>-3.836839715453304</v>
+        <v>-11.70336673206002</v>
       </c>
       <c r="H53" t="b">
         <v>0</v>
@@ -2934,7 +2934,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
@@ -2947,30 +2947,30 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Mushroom</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>6.856</v>
+        <v>0.6321</v>
       </c>
       <c r="E54" t="n">
-        <v>6.7014</v>
+        <v>0.5276</v>
       </c>
       <c r="F54" t="n">
-        <v>-0.1546000000000003</v>
+        <v>-0.1045</v>
       </c>
       <c r="G54" t="n">
-        <v>-2.254959159859981</v>
+        <v>-16.53219427305806</v>
       </c>
       <c r="H54" t="b">
         <v>0</v>
@@ -2994,30 +2994,30 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Mushroom</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>3.446302</v>
+        <v>0.544045</v>
       </c>
       <c r="E55" t="n">
-        <v>3.072402</v>
+        <v>0.433018</v>
       </c>
       <c r="F55" t="n">
-        <v>-0.3739000000000003</v>
+        <v>-0.111027</v>
       </c>
       <c r="G55" t="n">
-        <v>-10.84931036223756</v>
+        <v>-20.40768686413807</v>
       </c>
       <c r="H55" t="b">
         <v>0</v>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
@@ -3041,30 +3041,30 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Mushroom</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>8.513500000000001</v>
+        <v>0.538448</v>
       </c>
       <c r="E56" t="n">
-        <v>8.3148</v>
+        <v>0.394057</v>
       </c>
       <c r="F56" t="n">
-        <v>-0.1987000000000005</v>
+        <v>-0.144391</v>
       </c>
       <c r="G56" t="n">
-        <v>-2.333940212603518</v>
+        <v>-26.81614566309096</v>
       </c>
       <c r="H56" t="b">
         <v>0</v>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
@@ -3088,30 +3088,30 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Mushroom</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3.788867</v>
+        <v>1.1701</v>
       </c>
       <c r="E57" t="n">
-        <v>3.345442</v>
+        <v>1.0407</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.4434250000000004</v>
+        <v>-0.1294</v>
       </c>
       <c r="G57" t="n">
-        <v>-11.70336673206002</v>
+        <v>-11.05888385608067</v>
       </c>
       <c r="H57" t="b">
         <v>0</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
@@ -3140,25 +3140,25 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.6321</v>
+        <v>1.9831</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5276</v>
+        <v>1.8176</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.1045</v>
+        <v>-0.1655</v>
       </c>
       <c r="G58" t="n">
-        <v>-16.53219427305806</v>
+        <v>-8.345519640966163</v>
       </c>
       <c r="H58" t="b">
         <v>0</v>
@@ -3187,25 +3187,25 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.544045</v>
+        <v>0.615897</v>
       </c>
       <c r="E59" t="n">
-        <v>0.433018</v>
+        <v>0.486169</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.111027</v>
+        <v>-0.129728</v>
       </c>
       <c r="G59" t="n">
-        <v>-20.40768686413807</v>
+        <v>-21.06326220130964</v>
       </c>
       <c r="H59" t="b">
         <v>0</v>
@@ -3234,25 +3234,25 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.538448</v>
+        <v>9.373900000000001</v>
       </c>
       <c r="E60" t="n">
-        <v>0.394057</v>
+        <v>9.2433</v>
       </c>
       <c r="F60" t="n">
-        <v>-0.144391</v>
+        <v>-0.1306000000000012</v>
       </c>
       <c r="G60" t="n">
-        <v>-26.81614566309096</v>
+        <v>-1.393230139002989</v>
       </c>
       <c r="H60" t="b">
         <v>0</v>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
@@ -3281,25 +3281,25 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1.1701</v>
+        <v>0.698264</v>
       </c>
       <c r="E61" t="n">
-        <v>1.0407</v>
+        <v>0.539467</v>
       </c>
       <c r="F61" t="n">
-        <v>-0.1294</v>
+        <v>-0.158797</v>
       </c>
       <c r="G61" t="n">
-        <v>-11.05888385608067</v>
+        <v>-22.74168509331713</v>
       </c>
       <c r="H61" t="b">
         <v>0</v>
@@ -3310,7 +3310,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
@@ -3323,30 +3323,30 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mushroom</t>
+          <t>MAGIC</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.9831</v>
+        <v>1.432</v>
       </c>
       <c r="E62" t="n">
-        <v>1.8176</v>
+        <v>1.3078</v>
       </c>
       <c r="F62" t="n">
-        <v>-0.1655</v>
+        <v>-0.1241999999999999</v>
       </c>
       <c r="G62" t="n">
-        <v>-8.345519640966163</v>
+        <v>-8.67318435754189</v>
       </c>
       <c r="H62" t="b">
         <v>0</v>
@@ -3370,41 +3370,41 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mushroom</t>
+          <t>MAGIC</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.615897</v>
+        <v>1.25837</v>
       </c>
       <c r="E63" t="n">
-        <v>0.486169</v>
+        <v>2.000846</v>
       </c>
       <c r="F63" t="n">
-        <v>-0.129728</v>
+        <v>0.7424760000000001</v>
       </c>
       <c r="G63" t="n">
-        <v>-21.06326220130964</v>
+        <v>59.00299593919119</v>
       </c>
       <c r="H63" t="b">
         <v>0</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Hungarian worse (higher distance)</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>10000</v>
+        <v>19020</v>
       </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
@@ -3417,41 +3417,41 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mushroom</t>
+          <t>MAGIC</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9.373900000000001</v>
+        <v>1.948976</v>
       </c>
       <c r="E64" t="n">
-        <v>9.2433</v>
+        <v>2.490962</v>
       </c>
       <c r="F64" t="n">
-        <v>-0.1306000000000012</v>
+        <v>0.5419860000000001</v>
       </c>
       <c r="G64" t="n">
-        <v>-1.393230139002989</v>
+        <v>27.80875700880873</v>
       </c>
       <c r="H64" t="b">
         <v>0</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Hungarian worse (higher distance)</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>1000</v>
+        <v>19020</v>
       </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
@@ -3464,30 +3464,30 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Mushroom</t>
+          <t>MAGIC</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.698264</v>
+        <v>1.209</v>
       </c>
       <c r="E65" t="n">
-        <v>0.539467</v>
+        <v>1.1898</v>
       </c>
       <c r="F65" t="n">
-        <v>-0.158797</v>
+        <v>-0.01920000000000011</v>
       </c>
       <c r="G65" t="n">
-        <v>-22.74168509331713</v>
+        <v>-1.588089330024823</v>
       </c>
       <c r="H65" t="b">
         <v>0</v>
@@ -3498,7 +3498,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
@@ -3516,25 +3516,25 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.432</v>
+        <v>1.9498</v>
       </c>
       <c r="E66" t="n">
-        <v>1.3078</v>
+        <v>1.8741</v>
       </c>
       <c r="F66" t="n">
-        <v>-0.1241999999999999</v>
+        <v>-0.07569999999999988</v>
       </c>
       <c r="G66" t="n">
-        <v>-8.67318435754189</v>
+        <v>-3.882449481998147</v>
       </c>
       <c r="H66" t="b">
         <v>0</v>
@@ -3563,25 +3563,25 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.25837</v>
+        <v>2.43384</v>
       </c>
       <c r="E67" t="n">
-        <v>2.000846</v>
+        <v>3.383397</v>
       </c>
       <c r="F67" t="n">
-        <v>0.7424760000000001</v>
+        <v>0.949557</v>
       </c>
       <c r="G67" t="n">
-        <v>59.00299593919119</v>
+        <v>39.01476678828518</v>
       </c>
       <c r="H67" t="b">
         <v>0</v>
@@ -3610,36 +3610,36 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.948976</v>
+        <v>4.5721</v>
       </c>
       <c r="E68" t="n">
-        <v>2.490962</v>
+        <v>4.2848</v>
       </c>
       <c r="F68" t="n">
-        <v>0.5419860000000001</v>
+        <v>-0.2873000000000001</v>
       </c>
       <c r="G68" t="n">
-        <v>27.80875700880873</v>
+        <v>-6.283764572078478</v>
       </c>
       <c r="H68" t="b">
         <v>0</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Hungarian worse (higher distance)</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>19020</v>
+        <v>1000</v>
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
@@ -3657,36 +3657,36 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.209</v>
+        <v>2.200845</v>
       </c>
       <c r="E69" t="n">
-        <v>1.1898</v>
+        <v>3.055436</v>
       </c>
       <c r="F69" t="n">
-        <v>-0.01920000000000011</v>
+        <v>0.8545909999999997</v>
       </c>
       <c r="G69" t="n">
-        <v>-1.588089330024823</v>
+        <v>38.83013115417031</v>
       </c>
       <c r="H69" t="b">
         <v>0</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Hungarian worse (higher distance)</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>1000</v>
+        <v>19020</v>
       </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
@@ -3699,30 +3699,30 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MAGIC</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1.9498</v>
+        <v>0.35574</v>
       </c>
       <c r="E70" t="n">
-        <v>1.8741</v>
+        <v>0.297551</v>
       </c>
       <c r="F70" t="n">
-        <v>-0.07569999999999988</v>
+        <v>-0.05818899999999999</v>
       </c>
       <c r="G70" t="n">
-        <v>-3.882449481998147</v>
+        <v>-16.35717096756058</v>
       </c>
       <c r="H70" t="b">
         <v>0</v>
@@ -3746,30 +3746,30 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MAGIC</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2.43384</v>
+        <v>0.258434</v>
       </c>
       <c r="E71" t="n">
-        <v>3.383397</v>
+        <v>0.291262</v>
       </c>
       <c r="F71" t="n">
-        <v>0.949557</v>
+        <v>0.03282800000000002</v>
       </c>
       <c r="G71" t="n">
-        <v>39.01476678828518</v>
+        <v>12.70266296230373</v>
       </c>
       <c r="H71" t="b">
         <v>0</v>
@@ -3780,7 +3780,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>19020</v>
+        <v>5000</v>
       </c>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
@@ -3793,30 +3793,30 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MAGIC</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>4.5721</v>
+        <v>27.853218</v>
       </c>
       <c r="E72" t="n">
-        <v>4.2848</v>
+        <v>27.790041</v>
       </c>
       <c r="F72" t="n">
-        <v>-0.2873000000000001</v>
+        <v>-0.06317699999999959</v>
       </c>
       <c r="G72" t="n">
-        <v>-6.283764572078478</v>
+        <v>-0.2268211881298585</v>
       </c>
       <c r="H72" t="b">
         <v>0</v>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
@@ -3840,41 +3840,41 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MAGIC</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>2.200845</v>
+        <v>1.498572</v>
       </c>
       <c r="E73" t="n">
-        <v>3.055436</v>
+        <v>1.410562</v>
       </c>
       <c r="F73" t="n">
-        <v>0.8545909999999997</v>
+        <v>-0.08800999999999992</v>
       </c>
       <c r="G73" t="n">
-        <v>38.83013115417031</v>
+        <v>-5.872924357321497</v>
       </c>
       <c r="H73" t="b">
         <v>0</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Hungarian worse (higher distance)</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>19020</v>
+        <v>1000</v>
       </c>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>
@@ -3892,25 +3892,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.35574</v>
+        <v>1.607389</v>
       </c>
       <c r="E74" t="n">
-        <v>0.297551</v>
+        <v>1.468671</v>
       </c>
       <c r="F74" t="n">
-        <v>-0.05818899999999999</v>
+        <v>-0.1387179999999999</v>
       </c>
       <c r="G74" t="n">
-        <v>-16.35717096756058</v>
+        <v>-8.630020486640129</v>
       </c>
       <c r="H74" t="b">
         <v>0</v>
@@ -3939,32 +3939,32 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.258434</v>
+        <v>0.431625</v>
       </c>
       <c r="E75" t="n">
-        <v>0.291262</v>
+        <v>0.399805</v>
       </c>
       <c r="F75" t="n">
-        <v>0.03282800000000002</v>
+        <v>-0.03181999999999996</v>
       </c>
       <c r="G75" t="n">
-        <v>12.70266296230373</v>
+        <v>-7.372140167969873</v>
       </c>
       <c r="H75" t="b">
         <v>0</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Hungarian worse (higher distance)</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J75" t="n">
@@ -3986,25 +3986,25 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>27.853218</v>
+        <v>13.596022</v>
       </c>
       <c r="E76" t="n">
-        <v>27.790041</v>
+        <v>13.548747</v>
       </c>
       <c r="F76" t="n">
-        <v>-0.06317699999999959</v>
+        <v>-0.04727499999999907</v>
       </c>
       <c r="G76" t="n">
-        <v>-0.2268211881298585</v>
+        <v>-0.3477119998776044</v>
       </c>
       <c r="H76" t="b">
         <v>0</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
@@ -4033,25 +4033,25 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.498572</v>
+        <v>0.587039</v>
       </c>
       <c r="E77" t="n">
-        <v>1.410562</v>
+        <v>0.482782</v>
       </c>
       <c r="F77" t="n">
-        <v>-0.08800999999999992</v>
+        <v>-0.104257</v>
       </c>
       <c r="G77" t="n">
-        <v>-5.872924357321497</v>
+        <v>-17.75980812177726</v>
       </c>
       <c r="H77" t="b">
         <v>0</v>
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
@@ -4075,30 +4075,30 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Metro</t>
+          <t>OnlineShop</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.607389</v>
+        <v>1.94589</v>
       </c>
       <c r="E78" t="n">
-        <v>1.468671</v>
+        <v>1.816702</v>
       </c>
       <c r="F78" t="n">
-        <v>-0.1387179999999999</v>
+        <v>-0.1291879999999999</v>
       </c>
       <c r="G78" t="n">
-        <v>-8.630020486640129</v>
+        <v>-6.639018649563947</v>
       </c>
       <c r="H78" t="b">
         <v>0</v>
@@ -4122,30 +4122,30 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Metro</t>
+          <t>OnlineShop</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.431625</v>
+        <v>2.525588</v>
       </c>
       <c r="E79" t="n">
-        <v>0.399805</v>
+        <v>2.384212</v>
       </c>
       <c r="F79" t="n">
-        <v>-0.03181999999999996</v>
+        <v>-0.1413759999999997</v>
       </c>
       <c r="G79" t="n">
-        <v>-7.372140167969873</v>
+        <v>-5.597745950645938</v>
       </c>
       <c r="H79" t="b">
         <v>0</v>
@@ -4155,9 +4155,7 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J79" t="n">
-        <v>5000</v>
-      </c>
+      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
@@ -4169,30 +4167,30 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Metro</t>
+          <t>OnlineShop</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>13.596022</v>
+        <v>1.722005</v>
       </c>
       <c r="E80" t="n">
-        <v>13.548747</v>
+        <v>1.587593</v>
       </c>
       <c r="F80" t="n">
-        <v>-0.04727499999999907</v>
+        <v>-0.134412</v>
       </c>
       <c r="G80" t="n">
-        <v>-0.3477119998776044</v>
+        <v>-7.805552248686849</v>
       </c>
       <c r="H80" t="b">
         <v>0</v>
@@ -4202,9 +4200,7 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J80" t="n">
-        <v>1000</v>
-      </c>
+      <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
@@ -4216,30 +4212,30 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Metro</t>
+          <t>OnlineShop</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.587039</v>
+        <v>3.20519</v>
       </c>
       <c r="E81" t="n">
-        <v>0.482782</v>
+        <v>3.055943</v>
       </c>
       <c r="F81" t="n">
-        <v>-0.104257</v>
+        <v>-0.1492469999999999</v>
       </c>
       <c r="G81" t="n">
-        <v>-17.75980812177726</v>
+        <v>-4.65641662428748</v>
       </c>
       <c r="H81" t="b">
         <v>0</v>
@@ -4250,7 +4246,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
@@ -4268,25 +4264,25 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.94589</v>
+        <v>2.588096</v>
       </c>
       <c r="E82" t="n">
-        <v>1.816702</v>
+        <v>2.433242</v>
       </c>
       <c r="F82" t="n">
-        <v>-0.1291879999999999</v>
+        <v>-0.1548540000000003</v>
       </c>
       <c r="G82" t="n">
-        <v>-6.639018649563947</v>
+        <v>-5.983317465812716</v>
       </c>
       <c r="H82" t="b">
         <v>0</v>
@@ -4315,25 +4311,25 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>2.525588</v>
+        <v>1.712434</v>
       </c>
       <c r="E83" t="n">
-        <v>2.384212</v>
+        <v>1.567794</v>
       </c>
       <c r="F83" t="n">
-        <v>-0.1413759999999997</v>
+        <v>-0.1446400000000001</v>
       </c>
       <c r="G83" t="n">
-        <v>-5.597745950645938</v>
+        <v>-8.446456914543866</v>
       </c>
       <c r="H83" t="b">
         <v>0</v>
@@ -4360,25 +4356,25 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1.722005</v>
+        <v>5.801993</v>
       </c>
       <c r="E84" t="n">
-        <v>1.587593</v>
+        <v>5.638238</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.134412</v>
+        <v>-0.1637550000000001</v>
       </c>
       <c r="G84" t="n">
-        <v>-7.805552248686849</v>
+        <v>-2.822392236598701</v>
       </c>
       <c r="H84" t="b">
         <v>0</v>
@@ -4388,7 +4384,9 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="n">
+        <v>1000</v>
+      </c>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
@@ -4405,25 +4403,25 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>3.20519</v>
+        <v>1.741369</v>
       </c>
       <c r="E85" t="n">
-        <v>3.055943</v>
+        <v>1.581511</v>
       </c>
       <c r="F85" t="n">
-        <v>-0.1492469999999999</v>
+        <v>-0.1598580000000001</v>
       </c>
       <c r="G85" t="n">
-        <v>-4.65641662428748</v>
+        <v>-9.180018709417709</v>
       </c>
       <c r="H85" t="b">
         <v>0</v>
@@ -4433,9 +4431,7 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J85" t="n">
-        <v>1000</v>
-      </c>
+      <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
@@ -4447,30 +4443,30 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>OnlineShop</t>
+          <t>AirQuality</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>2.588096</v>
+        <v>1.7287</v>
       </c>
       <c r="E86" t="n">
-        <v>2.433242</v>
+        <v>1.6389</v>
       </c>
       <c r="F86" t="n">
-        <v>-0.1548540000000003</v>
+        <v>-0.08979999999999988</v>
       </c>
       <c r="G86" t="n">
-        <v>-5.983317465812716</v>
+        <v>-5.19465494302076</v>
       </c>
       <c r="H86" t="b">
         <v>0</v>
@@ -4494,30 +4490,30 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>OnlineShop</t>
+          <t>AirQuality</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1.712434</v>
+        <v>53.42266</v>
       </c>
       <c r="E87" t="n">
-        <v>1.567794</v>
+        <v>20.605003</v>
       </c>
       <c r="F87" t="n">
-        <v>-0.1446400000000001</v>
+        <v>-32.817657</v>
       </c>
       <c r="G87" t="n">
-        <v>-8.446456914543866</v>
+        <v>-61.43021893705779</v>
       </c>
       <c r="H87" t="b">
         <v>0</v>
@@ -4527,7 +4523,9 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="n">
+        <v>1000</v>
+      </c>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
@@ -4539,30 +4537,30 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>OnlineShop</t>
+          <t>AirQuality</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>5.801993</v>
+        <v>28.73888</v>
       </c>
       <c r="E88" t="n">
-        <v>5.638238</v>
+        <v>18.531944</v>
       </c>
       <c r="F88" t="n">
-        <v>-0.1637550000000001</v>
+        <v>-10.206936</v>
       </c>
       <c r="G88" t="n">
-        <v>-2.822392236598701</v>
+        <v>-35.51612310570211</v>
       </c>
       <c r="H88" t="b">
         <v>0</v>
@@ -4586,30 +4584,30 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>OnlineShop</t>
+          <t>AirQuality</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>1.741369</v>
+        <v>4.9184</v>
       </c>
       <c r="E89" t="n">
-        <v>1.581511</v>
+        <v>4.6189</v>
       </c>
       <c r="F89" t="n">
-        <v>-0.1598580000000001</v>
+        <v>-0.2995000000000001</v>
       </c>
       <c r="G89" t="n">
-        <v>-9.180018709417709</v>
+        <v>-6.089378659726743</v>
       </c>
       <c r="H89" t="b">
         <v>0</v>
@@ -4636,25 +4634,25 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1.7287</v>
+        <v>9.283799999999999</v>
       </c>
       <c r="E90" t="n">
-        <v>1.6389</v>
+        <v>9.02</v>
       </c>
       <c r="F90" t="n">
-        <v>-0.08979999999999988</v>
+        <v>-0.2637999999999998</v>
       </c>
       <c r="G90" t="n">
-        <v>-5.19465494302076</v>
+        <v>-2.841508864904455</v>
       </c>
       <c r="H90" t="b">
         <v>0</v>
@@ -4664,9 +4662,7 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J90" t="n">
-        <v>1000</v>
-      </c>
+      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
@@ -4683,25 +4679,25 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>53.42266</v>
+        <v>6.392</v>
       </c>
       <c r="E91" t="n">
-        <v>20.605003</v>
+        <v>6.1055</v>
       </c>
       <c r="F91" t="n">
-        <v>-32.817657</v>
+        <v>-0.2865000000000002</v>
       </c>
       <c r="G91" t="n">
-        <v>-61.43021893705779</v>
+        <v>-4.482165206508138</v>
       </c>
       <c r="H91" t="b">
         <v>0</v>
@@ -4725,30 +4721,30 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>28.73888</v>
+        <v>0.9112</v>
       </c>
       <c r="E92" t="n">
-        <v>18.531944</v>
+        <v>0.8489</v>
       </c>
       <c r="F92" t="n">
-        <v>-10.206936</v>
+        <v>-0.06230000000000002</v>
       </c>
       <c r="G92" t="n">
-        <v>-35.51612310570211</v>
+        <v>-6.837137840210714</v>
       </c>
       <c r="H92" t="b">
         <v>0</v>
@@ -4772,30 +4768,30 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>4.9184</v>
+        <v>3.345275</v>
       </c>
       <c r="E93" t="n">
-        <v>4.6189</v>
+        <v>3.145877</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.2995000000000001</v>
+        <v>-0.199398</v>
       </c>
       <c r="G93" t="n">
-        <v>-6.089378659726743</v>
+        <v>-5.960586199938719</v>
       </c>
       <c r="H93" t="b">
         <v>0</v>
@@ -4805,7 +4801,9 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" t="n">
+        <v>1000</v>
+      </c>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
@@ -4817,30 +4815,30 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>9.283799999999999</v>
+        <v>3.985879</v>
       </c>
       <c r="E94" t="n">
-        <v>9.02</v>
+        <v>3.685769</v>
       </c>
       <c r="F94" t="n">
-        <v>-0.2637999999999998</v>
+        <v>-0.3001100000000001</v>
       </c>
       <c r="G94" t="n">
-        <v>-2.841508864904455</v>
+        <v>-7.529330418710655</v>
       </c>
       <c r="H94" t="b">
         <v>0</v>
@@ -4850,7 +4848,9 @@
           <t>Hungarian better (lower distance)</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" t="n">
+        <v>1000</v>
+      </c>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
@@ -4862,30 +4862,30 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>15.87754573663957</v>
+        <v>3.6759</v>
       </c>
       <c r="E95" t="n">
-        <v>15.58214745304394</v>
+        <v>3.3891</v>
       </c>
       <c r="F95" t="n">
-        <v>-0.2953982835956328</v>
+        <v>-0.2867999999999999</v>
       </c>
       <c r="G95" t="n">
-        <v>-1.860478240752043</v>
+        <v>-7.802170896923201</v>
       </c>
       <c r="H95" t="b">
         <v>0</v>
@@ -4909,30 +4909,30 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>6.392</v>
+        <v>3.3377</v>
       </c>
       <c r="E96" t="n">
-        <v>6.1055</v>
+        <v>3.1203</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.2865000000000002</v>
+        <v>-0.2174</v>
       </c>
       <c r="G96" t="n">
-        <v>-4.482165206508138</v>
+        <v>-6.513467357761334</v>
       </c>
       <c r="H96" t="b">
         <v>0</v>
@@ -4956,30 +4956,30 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AirQuality</t>
+          <t>Concrete</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>17.04914586325495</v>
+        <v>5.242352</v>
       </c>
       <c r="E97" t="n">
-        <v>16.7797488635705</v>
+        <v>5.018745</v>
       </c>
       <c r="F97" t="n">
-        <v>-0.2693969996844494</v>
+        <v>-0.2236070000000003</v>
       </c>
       <c r="G97" t="n">
-        <v>-1.580120211564765</v>
+        <v>-4.265394616767442</v>
       </c>
       <c r="H97" t="b">
         <v>0</v>
@@ -5008,25 +5008,25 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.9112</v>
+        <v>1.7551</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8489</v>
+        <v>1.6227</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.06230000000000002</v>
+        <v>-0.1324000000000001</v>
       </c>
       <c r="G98" t="n">
-        <v>-6.837137840210714</v>
+        <v>-7.543729702011285</v>
       </c>
       <c r="H98" t="b">
         <v>0</v>
@@ -5055,25 +5055,25 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>3.345275</v>
+        <v>6.754965</v>
       </c>
       <c r="E99" t="n">
-        <v>3.145877</v>
+        <v>6.507187</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.199398</v>
+        <v>-0.2477780000000003</v>
       </c>
       <c r="G99" t="n">
-        <v>-5.960586199938719</v>
+        <v>-3.668087103338067</v>
       </c>
       <c r="H99" t="b">
         <v>0</v>
@@ -5097,30 +5097,30 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>3.985879</v>
+        <v>41.2109</v>
       </c>
       <c r="E100" t="n">
-        <v>3.685769</v>
+        <v>41.2089</v>
       </c>
       <c r="F100" t="n">
-        <v>-0.3001100000000001</v>
+        <v>-0.002000000000002444</v>
       </c>
       <c r="G100" t="n">
-        <v>-7.529330418710655</v>
+        <v>-0.004853084984803642</v>
       </c>
       <c r="H100" t="b">
         <v>0</v>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr"/>
@@ -5144,30 +5144,30 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>3.6759</v>
+        <v>18868.031041</v>
       </c>
       <c r="E101" t="n">
-        <v>3.3891</v>
+        <v>18868.030988</v>
       </c>
       <c r="F101" t="n">
-        <v>-0.2867999999999999</v>
+        <v>-5.299999975250103e-05</v>
       </c>
       <c r="G101" t="n">
-        <v>-7.802170896923201</v>
+        <v>-2.808984129681188e-07</v>
       </c>
       <c r="H101" t="b">
         <v>0</v>
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr"/>
@@ -5191,30 +5191,30 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>3.3377</v>
+        <v>21169.768599</v>
       </c>
       <c r="E102" t="n">
-        <v>3.1203</v>
+        <v>21169.768524</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.2174</v>
+        <v>-7.499999992433004e-05</v>
       </c>
       <c r="G102" t="n">
-        <v>-6.513467357761334</v>
+        <v>-3.542787894614627e-07</v>
       </c>
       <c r="H102" t="b">
         <v>0</v>
@@ -5225,7 +5225,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
@@ -5238,41 +5238,41 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>5.242352</v>
+        <v>23616.3467</v>
       </c>
       <c r="E103" t="n">
-        <v>5.018745</v>
+        <v>23616.3467</v>
       </c>
       <c r="F103" t="n">
-        <v>-0.2236070000000003</v>
+        <v>0</v>
       </c>
       <c r="G103" t="n">
-        <v>-4.265394616767442</v>
+        <v>0</v>
       </c>
       <c r="H103" t="b">
         <v>0</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Negligible / tie</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
@@ -5285,41 +5285,41 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>1.7551</v>
+        <v>21021.1892</v>
       </c>
       <c r="E104" t="n">
-        <v>1.6227</v>
+        <v>21021.1892</v>
       </c>
       <c r="F104" t="n">
-        <v>-0.1324000000000001</v>
+        <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>-7.543729702011285</v>
+        <v>0</v>
       </c>
       <c r="H104" t="b">
         <v>0</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Negligible / tie</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
@@ -5332,30 +5332,30 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Concrete</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>6.754965</v>
+        <v>45637.724946</v>
       </c>
       <c r="E105" t="n">
-        <v>6.507187</v>
+        <v>45637.724902</v>
       </c>
       <c r="F105" t="n">
-        <v>-0.2477780000000003</v>
+        <v>-4.400000034365803e-05</v>
       </c>
       <c r="G105" t="n">
-        <v>-3.668087103338067</v>
+        <v>-9.641146747722464e-08</v>
       </c>
       <c r="H105" t="b">
         <v>0</v>
@@ -5366,7 +5366,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>1000</v>
+        <v>768</v>
       </c>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
@@ -5384,32 +5384,32 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>41.2109</v>
+        <v>15946.4815</v>
       </c>
       <c r="E106" t="n">
-        <v>41.2089</v>
+        <v>15946.4815</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.002000000000002444</v>
+        <v>0</v>
       </c>
       <c r="G106" t="n">
-        <v>-0.004853084984803642</v>
+        <v>0</v>
       </c>
       <c r="H106" t="b">
         <v>0</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Hungarian better (lower distance)</t>
+          <t>Negligible / tie</t>
         </is>
       </c>
       <c r="J106" t="n">
@@ -5431,25 +5431,25 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>18868.031041</v>
+        <v>51117.382605</v>
       </c>
       <c r="E107" t="n">
-        <v>18868.030988</v>
+        <v>51117.382555</v>
       </c>
       <c r="F107" t="n">
-        <v>-5.299999975250103e-05</v>
+        <v>-5.000000237487257e-05</v>
       </c>
       <c r="G107" t="n">
-        <v>-2.808984129681188e-07</v>
+        <v>-9.781408950696522e-08</v>
       </c>
       <c r="H107" t="b">
         <v>0</v>
@@ -5473,30 +5473,30 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>GaussianCopula</t>
+          <t>ForestDiffusion</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Gaussian Copula</t>
+          <t>Forest Diffusion</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>21169.768599</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="E108" t="n">
-        <v>21169.768524</v>
+        <v>0.0771</v>
       </c>
       <c r="F108" t="n">
-        <v>-7.499999992433004e-05</v>
+        <v>-0.0001999999999999919</v>
       </c>
       <c r="G108" t="n">
-        <v>-3.542787894614627e-07</v>
+        <v>-0.2587322121604034</v>
       </c>
       <c r="H108" t="b">
         <v>0</v>
@@ -5507,7 +5507,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
@@ -5520,41 +5520,41 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>WGAN_GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>WGAN-GP</t>
+          <t>TVAE</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>23616.3467</v>
+        <v>16693.918272</v>
       </c>
       <c r="E109" t="n">
-        <v>23616.3467</v>
+        <v>16693.789109</v>
       </c>
       <c r="F109" t="n">
-        <v>0</v>
+        <v>-0.1291629999977886</v>
       </c>
       <c r="G109" t="n">
-        <v>0</v>
+        <v>-0.0007737129048632531</v>
       </c>
       <c r="H109" t="b">
         <v>0</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Negligible / tie</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J109" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
@@ -5567,41 +5567,41 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>CTABGAN</t>
+          <t>GaussianCopula</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>CTAB-GAN+</t>
+          <t>Gaussian Copula</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>21021.1892</v>
+        <v>16693.682733</v>
       </c>
       <c r="E110" t="n">
-        <v>21021.1892</v>
+        <v>16693.553751</v>
       </c>
       <c r="F110" t="n">
-        <v>0</v>
+        <v>-0.1289820000019972</v>
       </c>
       <c r="G110" t="n">
-        <v>0</v>
+        <v>-0.0007726395790847645</v>
       </c>
       <c r="H110" t="b">
         <v>0</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Negligible / tie</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
@@ -5614,30 +5614,30 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN_GP</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>CTGAN</t>
+          <t>WGAN-GP</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>45637.724946</v>
+        <v>1.4639</v>
       </c>
       <c r="E111" t="n">
-        <v>45637.724902</v>
+        <v>1.3965</v>
       </c>
       <c r="F111" t="n">
-        <v>-4.400000034365803e-05</v>
+        <v>-0.0673999999999999</v>
       </c>
       <c r="G111" t="n">
-        <v>-9.641146747722464e-08</v>
+        <v>-4.604139627023697</v>
       </c>
       <c r="H111" t="b">
         <v>0</v>
@@ -5648,7 +5648,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
@@ -5661,41 +5661,41 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTABGAN</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>TabDDPM</t>
+          <t>CTAB-GAN+</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>15946.4815</v>
+        <v>0.9013</v>
       </c>
       <c r="E112" t="n">
-        <v>15946.4815</v>
+        <v>0.8723</v>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>-0.02900000000000003</v>
       </c>
       <c r="G112" t="n">
-        <v>0</v>
+        <v>-3.217574614445804</v>
       </c>
       <c r="H112" t="b">
         <v>0</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Negligible / tie</t>
+          <t>Hungarian better (lower distance)</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
@@ -5708,30 +5708,30 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>RealEstate</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>CopulaGAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Copula GAN</t>
+          <t>CTGAN</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>51117.382605</v>
+        <v>16692.881415</v>
       </c>
       <c r="E113" t="n">
-        <v>51117.382555</v>
+        <v>16692.752234</v>
       </c>
       <c r="F113" t="n">
-        <v>-5.000000237487257e-05</v>
+        <v>-0.1291810000002442</v>
       </c>
       <c r="G113" t="n">
-        <v>-9.781408950696522e-08</v>
+        <v>-0.0007738687934616484</v>
       </c>
       <c r="H113" t="b">
         <v>0</v>
@@ -5742,7 +5742,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>768</v>
+        <v>414</v>
       </c>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
@@ -5760,25 +5760,25 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ForestDiffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Forest Diffusion</t>
+          <t>TabDDPM</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.9375</v>
       </c>
       <c r="E114" t="n">
-        <v>0.0771</v>
+        <v>0.8743</v>
       </c>
       <c r="F114" t="n">
-        <v>-0.0001999999999999919</v>
+        <v>-0.06320000000000003</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.2587322121604034</v>
+        <v>-6.741333333333338</v>
       </c>
       <c r="H114" t="b">
         <v>0</v>
@@ -5807,25 +5807,25 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>CopulaGAN</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>TVAE</t>
+          <t>Copula GAN</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>16693.918272</v>
+        <v>16693.963602</v>
       </c>
       <c r="E115" t="n">
-        <v>16693.789109</v>
+        <v>16693.834433</v>
       </c>
       <c r="F115" t="n">
-        <v>-0.1291629999977886</v>
+        <v>-0.1291689999998198</v>
       </c>
       <c r="G115" t="n">
-        <v>-0.0007737129048632531</v>
+        <v>-0.000773746745106985</v>
       </c>
       <c r="H115" t="b">
         <v>0</v>
@@ -5841,288 +5841,6 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>GaussianCopula</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Gaussian Copula</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
-        <v>16693.682733</v>
-      </c>
-      <c r="E116" t="n">
-        <v>16693.553751</v>
-      </c>
-      <c r="F116" t="n">
-        <v>-0.1289820000019972</v>
-      </c>
-      <c r="G116" t="n">
-        <v>-0.0007726395790847645</v>
-      </c>
-      <c r="H116" t="b">
-        <v>0</v>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J116" t="n">
-        <v>414</v>
-      </c>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>WGAN_GP</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>WGAN-GP</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>1.4639</v>
-      </c>
-      <c r="E117" t="n">
-        <v>1.3965</v>
-      </c>
-      <c r="F117" t="n">
-        <v>-0.0673999999999999</v>
-      </c>
-      <c r="G117" t="n">
-        <v>-4.604139627023697</v>
-      </c>
-      <c r="H117" t="b">
-        <v>0</v>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J117" t="n">
-        <v>414</v>
-      </c>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>CTABGAN</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>CTAB-GAN+</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
-        <v>0.9013</v>
-      </c>
-      <c r="E118" t="n">
-        <v>0.8723</v>
-      </c>
-      <c r="F118" t="n">
-        <v>-0.02900000000000003</v>
-      </c>
-      <c r="G118" t="n">
-        <v>-3.217574614445804</v>
-      </c>
-      <c r="H118" t="b">
-        <v>0</v>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J118" t="n">
-        <v>414</v>
-      </c>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>CTGAN</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>CTGAN</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
-        <v>16692.881415</v>
-      </c>
-      <c r="E119" t="n">
-        <v>16692.752234</v>
-      </c>
-      <c r="F119" t="n">
-        <v>-0.1291810000002442</v>
-      </c>
-      <c r="G119" t="n">
-        <v>-0.0007738687934616484</v>
-      </c>
-      <c r="H119" t="b">
-        <v>0</v>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J119" t="n">
-        <v>414</v>
-      </c>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>TabDDPM</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>TabDDPM</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="E120" t="n">
-        <v>0.8743</v>
-      </c>
-      <c r="F120" t="n">
-        <v>-0.06320000000000003</v>
-      </c>
-      <c r="G120" t="n">
-        <v>-6.741333333333338</v>
-      </c>
-      <c r="H120" t="b">
-        <v>0</v>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J120" t="n">
-        <v>414</v>
-      </c>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr">
-        <is>
-          <t>Not available in extracted results</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>RealEstate</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>CopulaGAN</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Copula GAN</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
-        <v>16693.963602</v>
-      </c>
-      <c r="E121" t="n">
-        <v>16693.834433</v>
-      </c>
-      <c r="F121" t="n">
-        <v>-0.1291689999998198</v>
-      </c>
-      <c r="G121" t="n">
-        <v>-0.000773746745106985</v>
-      </c>
-      <c r="H121" t="b">
-        <v>0</v>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>Hungarian better (lower distance)</t>
-        </is>
-      </c>
-      <c r="J121" t="n">
-        <v>414</v>
-      </c>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr">
         <is>
           <t>Not available in extracted results</t>
         </is>
@@ -6331,22 +6049,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>3.18677296584983</v>
+        <v>3.5259</v>
       </c>
       <c r="D7" t="n">
-        <v>2.890093722731807</v>
+        <v>3.302575</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.2966792431180231</v>
+        <v>-0.2233250000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1367471562866815</v>
+        <v>0.08840932737368087</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.2877500000000002</v>
+        <v>-0.2521</v>
       </c>
       <c r="H7" t="n">
         <v>100</v>
@@ -6499,22 +6217,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>17.17639144998682</v>
+        <v>17.41407333333333</v>
       </c>
       <c r="D13" t="n">
-        <v>11.6102679145768</v>
+        <v>10.08670783333333</v>
       </c>
       <c r="E13" t="n">
-        <v>-5.56612353541001</v>
+        <v>-7.327365499999999</v>
       </c>
       <c r="F13" t="n">
-        <v>11.54949334482794</v>
+        <v>13.10944605568217</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.2909491417978165</v>
+        <v>-0.2930000000000001</v>
       </c>
       <c r="H13" t="n">
         <v>100</v>
@@ -6705,25 +6423,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>2391.542782609838</v>
+        <v>2562.185114857143</v>
       </c>
       <c r="D3" t="n">
-        <v>2389.263592576157</v>
+        <v>2559.777961857143</v>
       </c>
       <c r="E3" t="n">
-        <v>-2.279190033680912</v>
+        <v>-2.407152999999826</v>
       </c>
       <c r="F3" t="n">
-        <v>8.452418160755425</v>
+        <v>8.756397965718179</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1413759999999997</v>
+        <v>-0.1352694999988941</v>
       </c>
       <c r="H3" t="n">
-        <v>86.66666666666667</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -6738,25 +6456,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="n">
-        <v>2549.061096494515</v>
+        <v>2730.982060785714</v>
       </c>
       <c r="D4" t="n">
-        <v>2548.259643721199</v>
+        <v>2730.134539</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.8014527733160101</v>
+        <v>-0.8475217857144232</v>
       </c>
       <c r="F4" t="n">
-        <v>2.611169436185693</v>
+        <v>2.703405078256759</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.144391</v>
+        <v>-0.1415509999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>93.33333333333333</v>
+        <v>92.85714285714286</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -6837,25 +6555,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>4191.713807989657</v>
+        <v>4835.102192538461</v>
       </c>
       <c r="D7" t="n">
-        <v>4191.588570994254</v>
+        <v>4835.011534</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1252369954025745</v>
+        <v>-0.09065853846158133</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3208004624114607</v>
+        <v>0.3314414587828434</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.2236070000000003</v>
+        <v>-0.1446400000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>93.33333333333333</v>
+        <v>92.30769230769231</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -6903,25 +6621,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>4559.27508912777</v>
+        <v>5259.146569692308</v>
       </c>
       <c r="D9" t="n">
-        <v>4559.128942848288</v>
+        <v>5259.031842461539</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1461462794822696</v>
+        <v>-0.1147272307693983</v>
       </c>
       <c r="F9" t="n">
-        <v>0.303774030532835</v>
+        <v>0.3139188068364924</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.2122929999999998</v>
+        <v>-0.1598580000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>93.33333333333333</v>
+        <v>92.30769230769231</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -7032,25 +6750,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D2" t="n">
-        <v>2228.795533469389</v>
+        <v>2345.711813517544</v>
       </c>
       <c r="E2" t="n">
-        <v>2228.311833309154</v>
+        <v>2345.220593429824</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.4837001602352213</v>
+        <v>-0.4912200877193183</v>
       </c>
       <c r="G2" t="n">
-        <v>3.121977584066546</v>
+        <v>3.203508345872733</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.1392589999999998</v>
+        <v>-0.133406</v>
       </c>
       <c r="I2" t="n">
-        <v>93.33333333333333</v>
+        <v>92.98245614035088</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -7058,13 +6776,13 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>6435</v>
+        <v>5772</v>
       </c>
       <c r="L2" t="n">
-        <v>2.438031880918587e-16</v>
+        <v>2.28491228901825e-15</v>
       </c>
       <c r="M2" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.7610983981693364</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -7072,7 +6790,7 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>2.438031880918587e-16</v>
+        <v>2.28491228901825e-15</v>
       </c>
     </row>
     <row r="3">
@@ -7142,25 +6860,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>2391.542782609838</v>
+        <v>2562.185114857143</v>
       </c>
       <c r="E4" t="n">
-        <v>2389.263592576157</v>
+        <v>2559.777961857143</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.279190033680912</v>
+        <v>-2.407152999999826</v>
       </c>
       <c r="G4" t="n">
-        <v>8.452418160755425</v>
+        <v>8.756397965718179</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1413759999999997</v>
+        <v>-0.1352694999988941</v>
       </c>
       <c r="I4" t="n">
-        <v>86.66666666666667</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -7168,13 +6886,13 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="L4" t="n">
-        <v>0.005126953125</v>
+        <v>0.00830078125</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7333333333333334</v>
+        <v>0.7142857142857142</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -7182,7 +6900,7 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.013427734375</v>
+        <v>0.02490234375</v>
       </c>
     </row>
     <row r="5">
@@ -7197,25 +6915,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>2549.061096494515</v>
+        <v>2730.982060785714</v>
       </c>
       <c r="E5" t="n">
-        <v>2548.259643721199</v>
+        <v>2730.134539</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.8014527733160101</v>
+        <v>-0.8475217857144232</v>
       </c>
       <c r="G5" t="n">
-        <v>2.611169436185693</v>
+        <v>2.703405078256759</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.144391</v>
+        <v>-0.1415509999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>93.33333333333333</v>
+        <v>92.85714285714286</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -7223,13 +6941,13 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00335693359375</v>
+        <v>0.00537109375</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7666666666666666</v>
+        <v>0.7523809523809524</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -7237,7 +6955,7 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>0.013427734375</v>
+        <v>0.021484375</v>
       </c>
     </row>
     <row r="6">
@@ -7362,25 +7080,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>4191.713807989657</v>
+        <v>4835.102192538461</v>
       </c>
       <c r="E8" t="n">
-        <v>4191.588570994254</v>
+        <v>4835.011534</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.1252369954025745</v>
+        <v>-0.09065853846158135</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3208004624114607</v>
+        <v>0.3314414587828435</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.2236070000000003</v>
+        <v>-0.1446400000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>93.33333333333333</v>
+        <v>92.30769230769231</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -7388,13 +7106,13 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="L8" t="n">
-        <v>0.004180908203125</v>
+        <v>0.0107421875</v>
       </c>
       <c r="M8" t="n">
-        <v>0.75</v>
+        <v>0.7142857142857142</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -7402,7 +7120,7 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>0.013427734375</v>
+        <v>0.02490234375</v>
       </c>
     </row>
     <row r="9">
@@ -7472,25 +7190,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" t="n">
-        <v>4559.27508912777</v>
+        <v>5259.146569692308</v>
       </c>
       <c r="E10" t="n">
-        <v>4559.128942848287</v>
+        <v>5259.031842461539</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1461462794822696</v>
+        <v>-0.1147272307693983</v>
       </c>
       <c r="G10" t="n">
-        <v>0.303774030532835</v>
+        <v>0.3139188068364924</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.2122929999999998</v>
+        <v>-0.1598580000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>93.33333333333333</v>
+        <v>92.30769230769231</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -7498,13 +7216,13 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="L10" t="n">
-        <v>0.004180908203125</v>
+        <v>0.0107421875</v>
       </c>
       <c r="M10" t="n">
-        <v>0.75</v>
+        <v>0.7142857142857142</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -7512,7 +7230,7 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>0.013427734375</v>
+        <v>0.02490234375</v>
       </c>
     </row>
     <row r="11">
@@ -7802,22 +7520,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>3.18677296584983</v>
+        <v>3.5259</v>
       </c>
       <c r="E16" t="n">
-        <v>2.890093722731807</v>
+        <v>3.302575</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.2966792431180231</v>
+        <v>-0.2233250000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1367471562866815</v>
+        <v>0.08840932737368087</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.2877500000000002</v>
+        <v>-0.2521</v>
       </c>
       <c r="I16" t="n">
         <v>100</v>
@@ -7828,10 +7546,10 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="L16" t="n">
-        <v>0.00390625</v>
+        <v>0.0625</v>
       </c>
       <c r="M16" t="n">
         <v>1</v>
@@ -7842,7 +7560,7 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>0.05859375</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="17">
@@ -8132,22 +7850,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D22" t="n">
-        <v>17.17639144998682</v>
+        <v>17.41407333333333</v>
       </c>
       <c r="E22" t="n">
-        <v>11.6102679145768</v>
+        <v>10.08670783333333</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.56612353541001</v>
+        <v>-7.327365499999999</v>
       </c>
       <c r="G22" t="n">
-        <v>11.54949334482794</v>
+        <v>13.10944605568216</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.2909491417978165</v>
+        <v>-0.2930000000000001</v>
       </c>
       <c r="I22" t="n">
         <v>100</v>
@@ -8158,10 +7876,10 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="L22" t="n">
-        <v>0.00390625</v>
+        <v>0.015625</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
@@ -8172,7 +7890,7 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>0.05859375</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="23">
@@ -8282,7 +8000,7 @@
         </is>
       </c>
       <c r="O24" t="n">
-        <v>0.0625</v>
+        <v>0.09375</v>
       </c>
     </row>
     <row r="25">
@@ -8351,9 +8069,129 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>generator</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Wine</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CTGAN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wine</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CopulaGAN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wine</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TVAE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Wine</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GaussianCopula</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AirQuality</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CTGAN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AirQuality</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CopulaGAN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>incomplete Mahalanobis methods available: ['Hungarian', 'One-to-One Greedy']</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8422,7 +8260,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -8432,7 +8270,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">

</xml_diff>